<commit_message>
Update: réponse Rufino RTVE + relances La Vanguardia et Kinotico
- RTVE Rufino Sanchez : répondu ×2, Gerardo & Javier en délibération
- La Vanguardia (Astrid) : 1ère relance 7 avr, 2ème relance 10 avr
- Kinotico (Iñaki/Matias) : 1ère relance 7 avr, 2ème relance 10 avr

https://claude.ai/code/session_01HYWxvMYnhgMLwDFxEAgpJK
</commit_message>
<xml_diff>
--- a/suivi_CP_Istoria_Lab.xlsx
+++ b/suivi_CP_Istoria_Lab.xlsx
@@ -1796,17 +1796,17 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>10/04/2026</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>En attente</t>
+          <t>En attente — 2e relance envoyée (BCN Film Fest / Sant Jordi)</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>✅ Répondu — transféré à Gerardo Sánchez &amp; Javier Sales</t>
+          <t>✅ Répondu (×2) — Gerardo &amp; Javier en délibération</t>
         </is>
       </c>
     </row>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
           <t>10/04/2026</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">

</xml_diff>